<commit_message>
📱 移动端优化 2026-02-24 23:57
</commit_message>
<xml_diff>
--- a/performance-dashboard/archive/交易表现_20260224.xlsx
+++ b/performance-dashboard/archive/交易表现_20260224.xlsx
@@ -685,26 +685,26 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>¥999,628.52</t>
+          <t>¥1,003,344.12</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>¥-371.48</t>
+          <t>¥+3,344.12</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>+0.33%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-1.33%</t>
+          <t>+11.09%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>-2.448</v>
+        <v>4.049</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -713,24 +713,24 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>71.4%</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>-0.0062%</t>
+          <t>0.0478%</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1.4424%</t>
+          <t>2.4877%</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -739,7 +739,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>20260213</t>
+          <t>20260224</t>
         </is>
       </c>
     </row>
@@ -2377,26 +2377,26 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>¥999,628.52</t>
+          <t>¥1,003,344.12</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>¥-371.48</t>
+          <t>¥+3,344.12</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>-0.04%</t>
+          <t>+0.33%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>-1.33%</t>
+          <t>+11.09%</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>-2.448</v>
+        <v>4.049</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -2405,24 +2405,24 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>71.4%</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>-0.0062%</t>
+          <t>0.0478%</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1.4424%</t>
+          <t>2.4877%</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>20260213</t>
+          <t>20260224</t>
         </is>
       </c>
     </row>

</xml_diff>